<commit_message>
Daily price update - 2026-06-14
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="EUR#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="EUR#,##0.00;[Red]-EUR#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +64,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -125,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -163,11 +169,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -555,7 +564,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-13 10:27</t>
+          <t>Last updated: 2026-06-14 10:48</t>
         </is>
       </c>
     </row>
@@ -641,7 +650,7 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>206</v>
@@ -662,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -767,159 +776,225 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F16" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G16" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="n">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F17" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G17" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
@@ -933,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1038,159 +1113,299 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F19" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G19" s="6" t="n">
         <v>206</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="n">
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F20" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G20" s="9" t="n">
         <v>206</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>329</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>

</xml_diff>

<commit_message>
Daily price update - 2026-06-15
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="EUR#,##0.00"/>
     <numFmt numFmtId="165" formatCode="EUR#,##0.00;[Red]-EUR#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +75,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -131,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -175,8 +180,14 @@
     <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -564,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-14 10:48</t>
+          <t>Last updated: 2026-06-15 13:54</t>
         </is>
       </c>
     </row>
@@ -671,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -809,193 +820,259 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G12" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n">
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F18" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G18" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="n">
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F19" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G19" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1008,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1146,267 +1223,333 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G12" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F16" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>206</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>208.33</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n">
+      <c r="E23" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F23" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G23" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-06-16
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-15 13:54</t>
+          <t>Last updated: 2026-06-16 12:52</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -853,226 +853,292 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="G13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G14" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F20" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G20" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="n">
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F21" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G21" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1085,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1256,300 +1322,366 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="G13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G14" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F18" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>208.33</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>206</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>209.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E25" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F25" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G25" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-06-17
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-16 12:52</t>
+          <t>Last updated: 2026-06-17 12:15</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -886,259 +886,325 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G14" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F22" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G22" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="n">
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F23" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G23" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1151,7 +1217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1355,334 +1421,400 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G14" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F20" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>209.5</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>206</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>210.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n">
+      <c r="E27" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F25" s="6" t="n">
+      <c r="F27" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G27" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-18
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,6 +187,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -575,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-17 12:15</t>
+          <t>Last updated: 2026-06-18 11:50</t>
         </is>
       </c>
     </row>
@@ -682,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -919,291 +922,357 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G15" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="G17" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F24" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G24" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="n">
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F25" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G25" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
@@ -1217,7 +1286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1454,367 +1523,433 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G15" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="G17" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F22" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>210.2</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>206</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>210.67</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>207.17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n">
+      <c r="E29" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F27" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="G29" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-19
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-18 11:50</t>
+          <t>Last updated: 2026-06-19 12:05</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -955,324 +955,390 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="G16" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G16" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="G18" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G18" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="G19" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="n">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G19" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="G20" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G26" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="n">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F25" s="9" t="n">
+      <c r="F27" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G25" s="9" t="n">
+      <c r="G27" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
@@ -1286,7 +1352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1556,400 +1622,466 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="G16" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G16" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="G18" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G18" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="G19" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="n">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G19" s="18" t="n">
+      <c r="G20" s="18" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F24" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>210.67</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>207.17</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="E31" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="F31" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G31" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A25:G25"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-20
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-19 12:05</t>
+          <t>Last updated: 2026-06-20 10:31</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -988,358 +988,424 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="G17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G17" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="G18" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="n">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="G19" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G19" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="G20" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G20" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="G21" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n">
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="F28" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G26" s="6" t="n">
+      <c r="G28" s="6" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="n">
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F29" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G27" s="9" t="n">
+      <c r="G29" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1352,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1655,433 +1721,499 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="G17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G17" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="G18" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="n">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="G19" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G19" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="G20" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G20" s="18" t="n">
+      <c r="G21" s="18" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F29" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G29" s="6" t="n">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>208</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>211.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>208.62</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E33" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F33" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G33" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-21
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-20 17:17</t>
+          <t>Last updated: 2026-06-21 11:15</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1120,490 +1120,556 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G20" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="G21" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n">
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n">
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="G25" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n">
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G26" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n">
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="n">
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F35" s="9" t="n">
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="9" t="n">
+      <c r="G37" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1616,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2051,565 +2117,631 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G20" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="G21" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G21" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n">
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G24" s="18" t="n">
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G25" s="18" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G26" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="F34" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>211.73</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <v>209.82</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>211.83</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>210.08</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E39" s="6" t="n">
+      <c r="E41" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="F41" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G41" s="6" t="n">
         <v>329</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-22
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-21 11:15</t>
+          <t>Last updated: 2026-06-22 13:34</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1153,523 +1153,589 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n">
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="G22" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n">
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G22" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="G23" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="G24" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="n">
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G24" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="G25" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n">
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G25" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="G26" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G26" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="G27" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="G28" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="G29" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n">
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G36" s="6" t="n">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="n">
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F37" s="9" t="n">
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="9" t="n">
+      <c r="G39" s="9" t="n">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-06-28
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-27 10:07</t>
+          <t>Last updated: 2026-06-28 10:26</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>166</v>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1351,722 +1351,969 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="G28" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="G29" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n">
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G39" s="16" t="n">
+      <c r="G40" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>365</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>406</v>
+      </c>
+      <c r="G52" s="16" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="n">
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="F57" s="6" t="n">
         <v>223</v>
       </c>
-      <c r="G48" s="6" t="n">
-        <v>215.78</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="G57" s="6" t="n">
+        <v>216.16</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="n">
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="F49" s="9" t="n">
+      <c r="F58" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="9" t="n">
-        <v>167.39</v>
+      <c r="G58" s="9" t="n">
+        <v>167.58</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>365</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>406</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>385.5</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2078,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2711,796 +2958,862 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n">
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G26" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n">
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G30" s="16" t="n">
+      <c r="G31" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="15" t="n">
+      <c r="G38" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F44" s="6" t="n">
+      <c r="F46" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F45" s="9" t="n">
+      <c r="F47" s="9" t="n">
         <v>280</v>
       </c>
-      <c r="G45" s="14" t="n">
+      <c r="G47" s="14" t="n">
         <v>-49</v>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="17" t="inlineStr">
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F50" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>212.18</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F51" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <v>208.88</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>212.22</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G53" s="9" t="n">
+        <v>208.72</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E52" s="6" t="n">
+      <c r="E54" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="F54" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G52" s="6" t="n">
+      <c r="G54" s="6" t="n">
         <v>304.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A50:G50"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A45:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-29
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-28 10:26</t>
+          <t>Last updated: 2026-06-29 12:32</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1384,935 +1384,1001 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>223</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G40" s="16" t="n">
+      <c r="G41" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="F50" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C54" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr">
+      <c r="D54" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G52" s="16" t="n">
+      <c r="G54" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="17" t="inlineStr">
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>216.16</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F58" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G58" s="9" t="n">
-        <v>167.58</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E59" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>333</v>
+        <v>223</v>
       </c>
       <c r="G59" s="6" t="n">
-        <v>333</v>
+        <v>216.5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>167.75</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C60" s="8" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="n">
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F60" s="9" t="n">
+      <c r="F62" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G60" s="9" t="n">
+      <c r="G62" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A49:G49"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2325,7 +2391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2991,829 +3057,895 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="G28" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G28" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="G29" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G31" s="16" t="n">
+      <c r="G32" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G39" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F46" s="6" t="n">
+      <c r="F48" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F47" s="9" t="n">
+      <c r="F49" s="9" t="n">
         <v>280</v>
       </c>
-      <c r="G47" s="14" t="n">
+      <c r="G49" s="14" t="n">
         <v>-49</v>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="G52" s="6" t="n">
-        <v>212.22</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F53" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <v>208.72</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>212.26</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>208.58</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E54" s="6" t="n">
+      <c r="E56" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="F56" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G54" s="6" t="n">
+      <c r="G56" s="6" t="n">
         <v>304.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A45:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-06-30
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-29 12:32</t>
+          <t>Last updated: 2026-06-30 10:55</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1417,968 +1417,1034 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G41" s="16" t="n">
+      <c r="G42" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F50" s="6" t="n">
+      <c r="F52" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C54" s="8" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D54" s="8" t="inlineStr">
+      <c r="D56" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G54" s="16" t="n">
+      <c r="G56" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="17" t="inlineStr">
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F59" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G59" s="6" t="n">
-        <v>216.5</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F60" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>167.75</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>333</v>
+        <v>223</v>
       </c>
       <c r="G61" s="6" t="n">
-        <v>333</v>
+        <v>216.81</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>167.9</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C62" s="8" t="inlineStr">
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="9" t="n">
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F62" s="9" t="n">
+      <c r="F64" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G62" s="9" t="n">
+      <c r="G64" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A51:G51"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2391,7 +2457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3090,861 +3156,960 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>223</v>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="G30" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G32" s="16" t="n">
+      <c r="G33" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="15" t="n">
+      <c r="G40" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="F50" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D51" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F49" s="9" t="n">
+      <c r="F51" s="9" t="n">
         <v>280</v>
       </c>
-      <c r="G49" s="14" t="n">
+      <c r="G51" s="14" t="n">
         <v>-49</v>
       </c>
     </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="17" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G52" s="18" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="n">
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="F57" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>212.8</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G54" s="6" t="n">
-        <v>212.26</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F55" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G55" s="9" t="n">
-        <v>208.58</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="12" t="inlineStr">
+      <c r="G58" s="9" t="n">
+        <v>208.45</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E56" s="6" t="n">
+      <c r="E59" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="F59" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G56" s="6" t="n">
-        <v>304.5</v>
+      <c r="G59" s="6" t="n">
+        <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A55:G55"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A49:G49"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-01
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-06-30 10:55</t>
+          <t>Last updated: 2026-07-01 11:22</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1450,1001 +1450,1067 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>223</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G42" s="16" t="n">
+      <c r="G43" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="F54" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C56" s="8" t="inlineStr">
+      <c r="C58" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr">
+      <c r="D58" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G56" s="16" t="n">
+      <c r="G58" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="17" t="inlineStr">
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F61" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G61" s="6" t="n">
-        <v>216.81</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F62" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G62" s="9" t="n">
-        <v>167.9</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>333</v>
+        <v>223</v>
       </c>
       <c r="G63" s="6" t="n">
-        <v>333</v>
+        <v>217.09</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>168.05</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C64" s="8" t="inlineStr">
+      <c r="C66" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="9" t="n">
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F64" s="9" t="n">
+      <c r="F66" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G64" s="9" t="n">
+      <c r="G66" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A53:G53"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2457,7 +2523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3189,927 +3255,993 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G30" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G31" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G33" s="16" t="n">
+      <c r="G34" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G41" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G51" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G53" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="F54" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G52" s="18" t="n">
+      <c r="G54" s="18" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="17" t="inlineStr">
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>212.8</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F58" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G58" s="9" t="n">
-        <v>208.45</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>213.29</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>208.33</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E59" s="6" t="n">
+      <c r="E61" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F59" s="6" t="n">
+      <c r="F61" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G59" s="6" t="n">
+      <c r="G61" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A55:G55"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A51:G51"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-02
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-01 11:22</t>
+          <t>Last updated: 2026-07-02 10:38</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1483,1034 +1483,1100 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G43" s="16" t="n">
+      <c r="G44" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="F56" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="G56" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C58" s="8" t="inlineStr">
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D58" s="8" t="inlineStr">
+      <c r="D60" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G58" s="16" t="n">
+      <c r="G60" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="17" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F63" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>217.09</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F64" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G64" s="9" t="n">
-        <v>168.05</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>333</v>
+        <v>223</v>
       </c>
       <c r="G65" s="6" t="n">
-        <v>333</v>
+        <v>217.35</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>168.17</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G67" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C66" s="8" t="inlineStr">
+      <c r="C68" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="9" t="n">
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F66" s="9" t="n">
+      <c r="F68" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G66" s="9" t="n">
+      <c r="G68" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2523,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3288,960 +3354,1026 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>223</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G34" s="16" t="n">
+      <c r="G35" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="15" t="n">
+      <c r="G42" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G53" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G55" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="F56" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G54" s="18" t="n">
+      <c r="G56" s="18" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="17" t="inlineStr">
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F59" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G59" s="6" t="n">
-        <v>213.29</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F60" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>208.33</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>213.73</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>213</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>208.23</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E61" s="6" t="n">
+      <c r="E63" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F61" s="6" t="n">
+      <c r="F63" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G61" s="6" t="n">
+      <c r="G63" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A53:G53"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A59:G59"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-03
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-02 10:38</t>
+          <t>Last updated: 2026-07-03 10:34</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1516,1067 +1516,1133 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>237</v>
+      </c>
+      <c r="G29" s="16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G44" s="16" t="n">
+      <c r="G45" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G55" s="16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="F58" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="G58" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="G61" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C60" s="8" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr">
+      <c r="D62" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G60" s="16" t="n">
+      <c r="G62" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="17" t="inlineStr">
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F65" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>217.35</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F66" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G66" s="9" t="n">
-        <v>168.17</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>333</v>
+        <v>237</v>
       </c>
       <c r="G67" s="6" t="n">
-        <v>333</v>
+        <v>218.17</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>168.88</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G69" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="9" t="n">
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F68" s="9" t="n">
+      <c r="F70" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G68" s="9" t="n">
+      <c r="G70" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A58:G58"/>
+    <mergeCell ref="A60:G60"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A65:G65"/>
+    <mergeCell ref="A57:G57"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2589,7 +2655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3387,993 +3453,1059 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>237</v>
+      </c>
+      <c r="G28" s="18" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="G33" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G35" s="16" t="n">
+      <c r="G36" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="15" t="n">
+      <c r="G43" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G53" s="18" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G55" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G57" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="F58" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G56" s="18" t="n">
+      <c r="G58" s="18" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="17" t="inlineStr">
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F61" s="6" t="n">
-        <v>223</v>
-      </c>
-      <c r="G61" s="6" t="n">
-        <v>213.73</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F62" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G62" s="9" t="n">
-        <v>208.23</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>237</v>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>214.74</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>209.04</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E63" s="6" t="n">
+      <c r="E65" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F63" s="6" t="n">
+      <c r="F65" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G63" s="6" t="n">
+      <c r="G65" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A59:G59"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-04
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -186,11 +186,11 @@
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-03 10:34</t>
+          <t>Last updated: 2026-07-04 10:08</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1549,1100 +1549,1166 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G45" s="16" t="n">
+      <c r="G46" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G55" s="16" t="n">
+      <c r="G56" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F58" s="6" t="n">
+      <c r="F60" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="G60" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="11" t="inlineStr">
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C62" s="8" t="inlineStr">
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D62" s="8" t="inlineStr">
+      <c r="D64" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G62" s="16" t="n">
+      <c r="G64" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="17" t="inlineStr">
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F67" s="6" t="n">
-        <v>237</v>
-      </c>
-      <c r="G67" s="6" t="n">
-        <v>218.17</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F68" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>168.88</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G69" s="6" t="n">
-        <v>333</v>
+        <v>219.28</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>169.52</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G71" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C70" s="8" t="inlineStr">
+      <c r="C72" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="9" t="n">
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F70" s="9" t="n">
+      <c r="F72" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G70" s="9" t="n">
+      <c r="G72" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A62:G62"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A65:G65"/>
-    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A59:G59"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2655,7 +2721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2822,7 +2888,7 @@
       <c r="F8" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="17" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3482,1030 +3548,1096 @@
       <c r="F28" s="6" t="n">
         <v>237</v>
       </c>
-      <c r="G28" s="18" t="n">
+      <c r="G28" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>237</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G33" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G36" s="16" t="n">
+      <c r="G37" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="15" t="n">
+      <c r="G44" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G53" s="18" t="n">
+      <c r="G54" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G57" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F58" s="6" t="n">
+      <c r="F60" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G58" s="18" t="n">
+      <c r="G60" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="17" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F63" s="6" t="n">
-        <v>237</v>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>214.74</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F64" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G64" s="9" t="n">
-        <v>209.04</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>237</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>215.67</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>209.79</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E65" s="6" t="n">
+      <c r="E67" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F65" s="6" t="n">
+      <c r="F67" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G65" s="6" t="n">
+      <c r="G67" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-05
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-04 10:08</t>
+          <t>Last updated: 2026-07-05 10:11</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1582,1133 +1582,1199 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G46" s="16" t="n">
+      <c r="G47" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G56" s="16" t="n">
+      <c r="G57" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F60" s="6" t="n">
+      <c r="F62" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="11" t="inlineStr">
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C64" s="8" t="inlineStr">
+      <c r="C66" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D64" s="8" t="inlineStr">
+      <c r="D66" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G64" s="16" t="n">
+      <c r="G66" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="18" t="inlineStr">
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="E70" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F69" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G69" s="6" t="n">
-        <v>219.28</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F70" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G70" s="9" t="n">
-        <v>169.52</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G71" s="6" t="n">
-        <v>333</v>
+        <v>220.31</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F72" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>170.12</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G73" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="9" t="n">
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F72" s="9" t="n">
+      <c r="F74" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G72" s="9" t="n">
+      <c r="G74" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A62:G62"/>
+    <mergeCell ref="A69:G69"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2721,7 +2787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3585,1059 +3651,1125 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G35" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G37" s="16" t="n">
+      <c r="G38" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="15" t="n">
+      <c r="G45" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G54" s="17" t="n">
+      <c r="G55" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G59" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G61" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F60" s="6" t="n">
+      <c r="F62" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G60" s="17" t="n">
+      <c r="G62" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="18" t="inlineStr">
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F65" s="6" t="n">
-        <v>237</v>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>215.67</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F66" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G66" s="9" t="n">
-        <v>209.79</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G67" s="6" t="n">
+        <v>216.88</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>210.48</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E67" s="6" t="n">
+      <c r="E69" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F67" s="6" t="n">
+      <c r="F69" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G67" s="6" t="n">
+      <c r="G69" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A65:G65"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-06
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-05 10:11</t>
+          <t>Last updated: 2026-07-06 12:03</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1615,1166 +1615,1232 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>-33</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G47" s="16" t="n">
+      <c r="G48" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G57" s="16" t="n">
+      <c r="G58" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F62" s="6" t="n">
+      <c r="F64" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="G67" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C66" s="8" t="inlineStr">
+      <c r="C68" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D66" s="8" t="inlineStr">
+      <c r="D68" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G66" s="16" t="n">
+      <c r="G68" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="18" t="inlineStr">
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F71" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G71" s="6" t="n">
-        <v>220.31</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F72" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G72" s="9" t="n">
-        <v>170.12</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G73" s="6" t="n">
-        <v>333</v>
+        <v>220.04</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>170.67</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G75" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr">
+      <c r="C76" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="9" t="n">
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F74" s="9" t="n">
+      <c r="F76" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G74" s="9" t="n">
+      <c r="G76" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A66:G66"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A64:G64"/>
-    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2787,7 +2853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3684,1092 +3750,1158 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G35" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G38" s="16" t="n">
+      <c r="G39" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="15" t="n">
+      <c r="G46" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G55" s="17" t="n">
+      <c r="G56" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G61" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G63" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F62" s="6" t="n">
+      <c r="F64" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G62" s="17" t="n">
+      <c r="G64" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="18" t="inlineStr">
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F67" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G67" s="6" t="n">
-        <v>216.88</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F68" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>210.48</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G69" s="6" t="n">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>211.12</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E69" s="6" t="n">
+      <c r="E71" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F69" s="6" t="n">
+      <c r="F71" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G69" s="6" t="n">
+      <c r="G71" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A67:G67"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A65:G65"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-07
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-06 12:03</t>
+          <t>Last updated: 2026-07-07 10:54</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1648,1199 +1648,1265 @@
         <v>-33</v>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>167</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>-46</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G48" s="16" t="n">
+      <c r="G49" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G58" s="16" t="n">
+      <c r="G59" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F64" s="6" t="n">
+      <c r="F66" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="G66" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D68" s="8" t="inlineStr">
+      <c r="D70" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G68" s="16" t="n">
+      <c r="G70" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="18" t="inlineStr">
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F72" s="3" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="n">
-        <v>213</v>
-      </c>
-      <c r="F73" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G73" s="6" t="n">
-        <v>220.04</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F74" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G74" s="9" t="n">
-        <v>170.67</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G75" s="6" t="n">
-        <v>333</v>
+        <v>218.14</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>171.18</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G77" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="9" t="n">
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F76" s="9" t="n">
+      <c r="F78" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G76" s="9" t="n">
+      <c r="G78" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A66:G66"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A71:G71"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A65:G65"/>
+    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A68:G68"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2853,7 +2919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3783,1125 +3849,1191 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G36" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="G37" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G39" s="16" t="n">
+      <c r="G40" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G47" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G56" s="17" t="n">
+      <c r="G57" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G63" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G65" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F64" s="6" t="n">
+      <c r="F66" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G64" s="17" t="n">
+      <c r="G66" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="18" t="inlineStr">
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="E70" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F69" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G69" s="6" t="n">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F70" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G70" s="9" t="n">
-        <v>211.12</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G71" s="6" t="n">
+        <v>219.04</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F72" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>211.7</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E71" s="6" t="n">
+      <c r="E73" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F71" s="6" t="n">
+      <c r="F73" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G71" s="6" t="n">
+      <c r="G73" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A69:G69"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-08
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-07 10:54</t>
+          <t>Last updated: 2026-07-08 10:15</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1681,1233 +1681,1299 @@
         <v>-46</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G49" s="16" t="n">
+      <c r="G50" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G59" s="16" t="n">
+      <c r="G60" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
+      <c r="B68" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F66" s="6" t="n">
+      <c r="F68" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="G68" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="11" t="inlineStr">
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G69" s="5" t="inlineStr">
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C70" s="8" t="inlineStr">
+      <c r="C72" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D70" s="8" t="inlineStr">
+      <c r="D72" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n">
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G70" s="16" t="n">
+      <c r="G72" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="18" t="inlineStr">
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G74" s="3" t="inlineStr">
+      <c r="G76" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F75" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G75" s="6" t="n">
-        <v>218.14</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F76" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>171.18</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G77" s="6" t="n">
-        <v>333</v>
+        <v>216.38</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>171.66</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G79" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C78" s="8" t="inlineStr">
+      <c r="C80" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E78" s="9" t="n">
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F78" s="9" t="n">
+      <c r="F80" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G78" s="9" t="n">
+      <c r="G80" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A70:G70"/>
+    <mergeCell ref="A67:G67"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A65:G65"/>
-    <mergeCell ref="A73:G73"/>
-    <mergeCell ref="A68:G68"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A75:G75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2919,7 +2985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3882,1158 +3948,1224 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G40" s="16" t="n">
+      <c r="G41" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
+      <c r="G48" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G57" s="17" t="n">
+      <c r="G58" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G65" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
+      <c r="B68" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F66" s="6" t="n">
+      <c r="F68" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G66" s="17" t="n">
+      <c r="G68" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="18" t="inlineStr">
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F71" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G71" s="6" t="n">
-        <v>219.04</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F72" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G72" s="9" t="n">
-        <v>211.7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G73" s="6" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>212.25</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E73" s="6" t="n">
+      <c r="E75" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F73" s="6" t="n">
+      <c r="F75" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G73" s="6" t="n">
+      <c r="G75" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A65:G65"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-09
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-08 10:15</t>
+          <t>Last updated: 2026-07-09 10:53</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1714,1266 +1714,1332 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>167</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G50" s="16" t="n">
+      <c r="G51" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G60" s="16" t="n">
+      <c r="G61" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E70" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F68" s="6" t="n">
+      <c r="F70" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="n">
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr">
+      <c r="D74" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n">
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G72" s="16" t="n">
+      <c r="G74" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="18" t="inlineStr">
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="F78" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G76" s="3" t="inlineStr">
+      <c r="G78" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F77" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G77" s="6" t="n">
-        <v>216.38</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E78" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F78" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G78" s="9" t="n">
-        <v>171.66</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G79" s="6" t="n">
-        <v>333</v>
+        <v>214.73</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>172.1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G81" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B82" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C80" s="8" t="inlineStr">
+      <c r="C82" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E80" s="9" t="n">
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F80" s="9" t="n">
+      <c r="F82" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G80" s="9" t="n">
+      <c r="G82" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A70:G70"/>
-    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A77:G77"/>
+    <mergeCell ref="A69:G69"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A72:G72"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A75:G75"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2985,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3981,1191 +4047,1257 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="G39" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G41" s="16" t="n">
+      <c r="G42" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="15" t="n">
+      <c r="G49" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G58" s="17" t="n">
+      <c r="G59" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G67" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G69" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E70" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F68" s="6" t="n">
+      <c r="F70" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G68" s="17" t="n">
+      <c r="G70" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="18" t="inlineStr">
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F72" s="3" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F73" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G73" s="6" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F74" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G74" s="9" t="n">
-        <v>212.25</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G75" s="6" t="n">
+        <v>220.9</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>212.76</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B75" s="5" t="inlineStr">
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E75" s="6" t="n">
+      <c r="E77" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F75" s="6" t="n">
+      <c r="F77" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G75" s="6" t="n">
+      <c r="G77" s="6" t="n">
         <v>301</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A67:G67"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A65:G65"/>
-    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A73:G73"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-10
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-09 10:53</t>
+          <t>Last updated: 2026-07-10 10:51</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1747,1299 +1747,1365 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G51" s="16" t="n">
+      <c r="G52" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G61" s="16" t="n">
+      <c r="G62" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G64" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G66" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="G67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F70" s="6" t="n">
+      <c r="F72" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G70" s="5" t="inlineStr">
+      <c r="G72" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="11" t="inlineStr">
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="n">
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G73" s="5" t="inlineStr">
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B74" s="13" t="inlineStr">
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr">
+      <c r="C76" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D74" s="8" t="inlineStr">
+      <c r="D76" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="n">
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G74" s="16" t="n">
+      <c r="G76" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="18" t="inlineStr">
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F78" s="3" t="inlineStr">
+      <c r="F80" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G78" s="3" t="inlineStr">
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F79" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G79" s="6" t="n">
-        <v>214.73</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E80" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F80" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G80" s="9" t="n">
-        <v>172.1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F81" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G81" s="6" t="n">
-        <v>333</v>
+        <v>213.19</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F82" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>172.52</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G83" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B84" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C82" s="8" t="inlineStr">
+      <c r="C84" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D82" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E82" s="9" t="n">
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F82" s="9" t="n">
+      <c r="F84" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G82" s="9" t="n">
+      <c r="G84" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A77:G77"/>
-    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A74:G74"/>
+    <mergeCell ref="A79:G79"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A72:G72"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3051,7 +3117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4080,1225 +4146,1324 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G42" s="16" t="n">
+      <c r="G43" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
+      <c r="G50" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G59" s="17" t="n">
+      <c r="G60" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G69" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F70" s="6" t="n">
+      <c r="F72" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G70" s="17" t="n">
+      <c r="G72" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="18" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="G73" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G74" s="3" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="6" t="n">
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="F75" s="6" t="n">
+      <c r="F78" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G75" s="6" t="n">
-        <v>220.9</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="9" t="n">
+      <c r="G78" s="6" t="n">
+        <v>221.73</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="F76" s="9" t="n">
+      <c r="F79" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G76" s="9" t="n">
-        <v>212.76</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="12" t="inlineStr">
+      <c r="G79" s="9" t="n">
+        <v>213.23</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E77" s="6" t="n">
+      <c r="E80" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F77" s="6" t="n">
+      <c r="F80" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G77" s="6" t="n">
-        <v>301</v>
+      <c r="G80" s="6" t="n">
+        <v>299.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A69:G69"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A76:G76"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-07-11
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-10 10:51</t>
+          <t>Last updated: 2026-07-11 09:27</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1780,1331 +1780,1397 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>174</v>
+      </c>
+      <c r="G37" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G52" s="16" t="n">
+      <c r="G53" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G62" s="16" t="n">
+      <c r="G63" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G67" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="G68" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="G69" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="G70" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B72" s="12" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F72" s="6" t="n">
+      <c r="F74" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F75" s="6" t="n">
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G75" s="5" t="inlineStr">
+      <c r="G77" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B76" s="13" t="inlineStr">
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D76" s="8" t="inlineStr">
+      <c r="D78" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F76" s="9" t="n">
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G76" s="16" t="n">
+      <c r="G78" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="18" t="inlineStr">
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F80" s="3" t="inlineStr">
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G80" s="3" t="inlineStr">
+      <c r="G82" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F81" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G81" s="6" t="n">
-        <v>213.19</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B82" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D82" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E82" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F82" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G82" s="9" t="n">
-        <v>172.52</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E83" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G83" s="6" t="n">
-        <v>333</v>
+        <v>211.97</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>172.91</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G85" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B86" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D84" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E84" s="9" t="n">
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F84" s="9" t="n">
+      <c r="F86" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G84" s="9" t="n">
+      <c r="G86" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A74:G74"/>
-    <mergeCell ref="A79:G79"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A76:G76"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="A73:G73"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3117,7 +3183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4179,1084 +4245,1082 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="G41" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G43" s="16" t="n">
+      <c r="G44" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G50" s="15" t="n">
+      <c r="G51" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G60" s="17" t="n">
+      <c r="G61" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G64" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="G67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G71" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
@@ -5280,190 +5344,258 @@
         </is>
       </c>
       <c r="F72" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G72" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G73" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G74" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B73" s="13" t="inlineStr">
+      <c r="B75" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C73" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr">
+      <c r="D75" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E73" s="8" t="inlineStr">
+      <c r="E75" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F73" s="9" t="n">
+      <c r="F75" s="9" t="n">
         <v>294</v>
       </c>
-      <c r="G73" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="18" t="inlineStr">
+      <c r="G75" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F77" s="3" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G79" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F78" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G78" s="6" t="n">
-        <v>221.73</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B79" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E79" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F79" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G79" s="9" t="n">
-        <v>213.23</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <v>222.52</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F81" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G81" s="9" t="n">
+        <v>213.68</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B80" s="5" t="inlineStr">
+      <c r="B82" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="D82" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E80" s="6" t="n">
+      <c r="E82" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F80" s="6" t="n">
+      <c r="F82" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G80" s="6" t="n">
+      <c r="G82" s="6" t="n">
         <v>299.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A78:G78"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-07-12
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-11 09:27</t>
+          <t>Last updated: 2026-07-12 09:49</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1813,1365 +1813,1431 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G53" s="16" t="n">
+      <c r="G54" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G63" s="16" t="n">
+      <c r="G64" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G64" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G66" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="G67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G68" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G69" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="G70" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="n">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G70" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="G71" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G71" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="G72" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G73" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B74" s="12" t="inlineStr">
+      <c r="B76" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E74" s="5" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F74" s="6" t="n">
+      <c r="F76" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G74" s="5" t="inlineStr">
+      <c r="G76" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="11" t="inlineStr">
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr">
+      <c r="B79" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="n">
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G77" s="5" t="inlineStr">
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B78" s="13" t="inlineStr">
+      <c r="B80" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C78" s="8" t="inlineStr">
+      <c r="C80" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D78" s="8" t="inlineStr">
+      <c r="D80" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="n">
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G78" s="16" t="n">
+      <c r="G80" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="18" t="inlineStr">
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
+      <c r="E84" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F82" s="3" t="inlineStr">
+      <c r="F84" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G82" s="3" t="inlineStr">
+      <c r="G84" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E83" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F83" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G83" s="6" t="n">
-        <v>211.97</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B84" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D84" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E84" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F84" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G84" s="9" t="n">
-        <v>172.91</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E85" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G85" s="6" t="n">
-        <v>333</v>
+        <v>210.82</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F86" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>173.27</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G87" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B88" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
+      <c r="C88" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D86" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E86" s="9" t="n">
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F86" s="9" t="n">
+      <c r="F88" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G86" s="9" t="n">
+      <c r="G88" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A78:G78"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A81:G81"/>
-    <mergeCell ref="A73:G73"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A75:G75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3183,7 +3249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4278,1117 +4344,1115 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G44" s="16" t="n">
+      <c r="G45" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G51" s="15" t="n">
+      <c r="G52" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G61" s="17" t="n">
+      <c r="G62" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="G68" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="G69" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="G70" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B72" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G73" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -5412,189 +5476,257 @@
         </is>
       </c>
       <c r="F74" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G74" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G75" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G76" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
+      <c r="B77" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D75" s="8" t="inlineStr">
+      <c r="D77" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E75" s="8" t="inlineStr">
+      <c r="E77" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F75" s="9" t="n">
+      <c r="F77" s="9" t="n">
         <v>294</v>
       </c>
-      <c r="G75" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="18" t="inlineStr">
+      <c r="G77" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr">
+      <c r="C81" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr">
+      <c r="D81" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E79" s="3" t="inlineStr">
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F79" s="3" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G79" s="3" t="inlineStr">
+      <c r="G81" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F80" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G80" s="6" t="n">
-        <v>222.52</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B81" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E81" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F81" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G81" s="9" t="n">
-        <v>213.68</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F82" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G82" s="6" t="n">
+        <v>223.25</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F83" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>214.09</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B82" s="5" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D82" s="5" t="inlineStr">
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E82" s="6" t="n">
+      <c r="E84" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F82" s="6" t="n">
+      <c r="F84" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G82" s="6" t="n">
+      <c r="G84" s="6" t="n">
         <v>299.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A78:G78"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A73:G73"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-13
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-12 09:49</t>
+          <t>Last updated: 2026-07-13 11:09</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1846,1398 +1846,1464 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>174</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G42" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G43" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>166</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G54" s="16" t="n">
+      <c r="G55" s="16" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>171</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G64" s="16" t="n">
+      <c r="G65" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G67" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="G68" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="G69" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="G70" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G70" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="G71" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="n">
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G71" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="G72" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G72" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+      <c r="G73" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="n">
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="G73" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
+      <c r="G74" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G75" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="5" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="B78" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="D78" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E76" s="5" t="inlineStr">
+      <c r="E78" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F76" s="6" t="n">
+      <c r="F78" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G76" s="5" t="inlineStr">
+      <c r="G78" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="11" t="inlineStr">
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="5" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B79" s="12" t="inlineStr">
+      <c r="B81" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F79" s="6" t="n">
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G79" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B80" s="13" t="inlineStr">
+      <c r="B82" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C80" s="8" t="inlineStr">
+      <c r="C82" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D80" s="8" t="inlineStr">
+      <c r="D82" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F80" s="9" t="n">
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G80" s="16" t="n">
+      <c r="G82" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="18" t="inlineStr">
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E84" s="3" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F84" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G84" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E85" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="F85" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G85" s="6" t="n">
-        <v>210.82</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D86" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E86" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="F86" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G86" s="9" t="n">
-        <v>173.27</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>17:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E87" s="6" t="n">
-        <v>333</v>
+        <v>167</v>
       </c>
       <c r="F87" s="6" t="n">
-        <v>333</v>
+        <v>246</v>
       </c>
       <c r="G87" s="6" t="n">
-        <v>333</v>
+        <v>209.74</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="13" t="inlineStr">
         <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="F88" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>173.82</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G89" s="6" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C88" s="8" t="inlineStr">
+      <c r="C90" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D88" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E88" s="9" t="n">
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="n">
         <v>365</v>
       </c>
-      <c r="F88" s="9" t="n">
+      <c r="F90" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G88" s="9" t="n">
+      <c r="G90" s="9" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A78:G78"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="A77:G77"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A85:G85"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A75:G75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3249,7 +3315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4377,1150 +4443,1148 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G41" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G45" s="16" t="n">
+      <c r="G46" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G52" s="15" t="n">
+      <c r="G53" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G62" s="17" t="n">
+      <c r="G63" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G64" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="G67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="G70" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="n">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G70" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="G71" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G71" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="G72" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G73" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B74" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F74" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B75" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G75" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
@@ -5544,190 +5608,258 @@
         </is>
       </c>
       <c r="F76" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G76" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G77" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G78" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B77" s="13" t="inlineStr">
+      <c r="B79" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D77" s="8" t="inlineStr">
+      <c r="D79" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E77" s="8" t="inlineStr">
+      <c r="E79" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F77" s="9" t="n">
+      <c r="F79" s="9" t="n">
         <v>294</v>
       </c>
-      <c r="G77" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="18" t="inlineStr">
+      <c r="G79" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr">
+      <c r="C83" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="E83" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F81" s="3" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G81" s="3" t="inlineStr">
+      <c r="G83" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E82" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F82" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G82" s="6" t="n">
-        <v>223.25</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E83" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F83" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G83" s="9" t="n">
-        <v>214.09</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G84" s="6" t="n">
+        <v>223.94</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F85" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>214.48</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B84" s="5" t="inlineStr">
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E84" s="6" t="n">
+      <c r="E86" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F84" s="6" t="n">
+      <c r="F86" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G84" s="6" t="n">
+      <c r="G86" s="6" t="n">
         <v>299.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A80:G80"/>
-    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A82:G82"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A75:G75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-07-15
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-14 09:56</t>
+          <t>Last updated: 2026-07-15 10:01</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>166</v>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1912,151 +1912,92 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>247</v>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -2082,14 +2023,16 @@
       <c r="F47" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
@@ -2122,7 +2065,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -2155,7 +2098,7 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
@@ -2188,7 +2131,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -2221,7 +2164,7 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
@@ -2254,7 +2197,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -2287,7 +2230,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -2320,7 +2263,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -2353,7 +2296,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -2377,16 +2320,16 @@
         </is>
       </c>
       <c r="F56" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G56" s="16" t="n">
-        <v>5</v>
+        <v>166</v>
+      </c>
+      <c r="G56" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -2410,7 +2353,7 @@
         </is>
       </c>
       <c r="F57" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G57" s="15" t="n">
         <v>0</v>
@@ -2419,7 +2362,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -2443,7 +2386,7 @@
         </is>
       </c>
       <c r="F58" s="9" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G58" s="14" t="n">
         <v>0</v>
@@ -2452,7 +2395,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -2476,7 +2419,7 @@
         </is>
       </c>
       <c r="F59" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G59" s="15" t="n">
         <v>0</v>
@@ -2485,7 +2428,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -2511,14 +2454,14 @@
       <c r="F60" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
+      <c r="G60" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -2551,7 +2494,7 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -2584,7 +2527,7 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -2617,7 +2560,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -2650,7 +2593,7 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2683,7 +2626,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -2707,16 +2650,16 @@
         </is>
       </c>
       <c r="F66" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G66" s="16" t="n">
-        <v>14</v>
+        <v>171</v>
+      </c>
+      <c r="G66" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2740,7 +2683,7 @@
         </is>
       </c>
       <c r="F67" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G67" s="15" t="n">
         <v>0</v>
@@ -2749,7 +2692,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -2773,7 +2716,7 @@
         </is>
       </c>
       <c r="F68" s="9" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G68" s="14" t="n">
         <v>0</v>
@@ -2782,7 +2725,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2806,7 +2749,7 @@
         </is>
       </c>
       <c r="F69" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G69" s="15" t="n">
         <v>0</v>
@@ -2815,7 +2758,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -2841,14 +2784,14 @@
       <c r="F70" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G70" s="14" t="n">
-        <v>0</v>
+      <c r="G70" s="16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2881,7 +2824,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -2914,7 +2857,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2947,7 +2890,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -2980,7 +2923,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -3013,7 +2956,7 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -3037,339 +2980,536 @@
         </is>
       </c>
       <c r="F76" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="G76" s="16" t="n">
-        <v>7</v>
+        <v>185</v>
+      </c>
+      <c r="G76" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G77" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="G78" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="G79" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G80" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="n">
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n">
         <v>192</v>
       </c>
-      <c r="G77" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="G81" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G82" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="5" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B80" s="12" t="inlineStr">
+      <c r="B85" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="D85" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E80" s="5" t="inlineStr">
+      <c r="E85" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F80" s="6" t="n">
+      <c r="F85" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="G80" s="5" t="inlineStr">
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="5" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B83" s="12" t="inlineStr">
+      <c r="B88" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F83" s="6" t="n">
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="G88" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B84" s="13" t="inlineStr">
+      <c r="B89" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D84" s="8" t="inlineStr">
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F84" s="9" t="n">
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G84" s="16" t="n">
+      <c r="G89" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="18" t="inlineStr">
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B93" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="C93" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr">
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F88" s="3" t="inlineStr">
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G88" s="3" t="inlineStr">
+      <c r="G93" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E89" s="6" t="n">
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="n">
         <v>167</v>
       </c>
-      <c r="F89" s="6" t="n">
+      <c r="F94" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G89" s="6" t="n">
-        <v>208.71</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D90" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E90" s="9" t="n">
+      <c r="G94" s="6" t="n">
+        <v>207.92</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>247</v>
+      </c>
+      <c r="F95" s="9" t="n">
+        <v>247</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="F90" s="9" t="n">
+      <c r="F96" s="6" t="n">
         <v>192</v>
       </c>
-      <c r="G90" s="9" t="n">
-        <v>174.34</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="12" t="inlineStr">
+      <c r="G96" s="6" t="n">
+        <v>174.83</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="B97" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C97" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D97" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E91" s="6" t="n">
+      <c r="E97" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="F91" s="6" t="n">
+      <c r="F97" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="G91" s="6" t="n">
+      <c r="G97" s="9" t="n">
         <v>333</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="13" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C92" s="8" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E92" s="9" t="n">
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="F92" s="9" t="n">
+      <c r="F98" s="6" t="n">
         <v>406</v>
       </c>
-      <c r="G92" s="9" t="n">
+      <c r="G98" s="6" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="A84:G84"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A79:G79"/>
     <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A92:G92"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A82:G82"/>
+    <mergeCell ref="A43:G43"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3381,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4575,1216 +4715,1214 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n">
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G44" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="G45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G47" s="16" t="n">
+      <c r="G48" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G54" s="15" t="n">
+      <c r="G55" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="G57" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G64" s="17" t="n">
+      <c r="G65" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="G67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="G70" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="n">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G70" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="G71" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G71" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
+      <c r="G72" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B72" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="n">
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G72" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="G73" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="n">
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G73" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+      <c r="G74" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B74" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F74" s="6" t="n">
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G74" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="G75" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="n">
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G75" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="11" t="inlineStr">
+      <c r="G76" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G77" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B78" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F78" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G78" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F79" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G79" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -5808,16 +5946,18 @@
         </is>
       </c>
       <c r="F80" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G80" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
@@ -5841,189 +5981,255 @@
         </is>
       </c>
       <c r="F81" s="9" t="n">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>0</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G82" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="G83" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B82" s="12" t="inlineStr">
+      <c r="B84" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D82" s="5" t="inlineStr">
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E82" s="5" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F82" s="6" t="n">
+      <c r="F84" s="6" t="n">
         <v>295</v>
       </c>
-      <c r="G82" s="17" t="n">
+      <c r="G84" s="17" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="18" t="inlineStr">
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr">
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr">
+      <c r="D88" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E86" s="3" t="inlineStr">
+      <c r="E88" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F86" s="3" t="inlineStr">
+      <c r="F88" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G86" s="3" t="inlineStr">
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F87" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G87" s="6" t="n">
-        <v>224.59</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D88" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E88" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F88" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G88" s="9" t="n">
-        <v>214.85</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>246</v>
+      </c>
+      <c r="G89" s="6" t="n">
+        <v>225.2</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F90" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>215.2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E89" s="6" t="n">
+      <c r="E91" s="6" t="n">
         <v>280</v>
       </c>
-      <c r="F89" s="6" t="n">
+      <c r="F91" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G89" s="6" t="n">
+      <c r="G91" s="6" t="n">
         <v>298.4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A77:G77"/>
+    <mergeCell ref="A79:G79"/>
+    <mergeCell ref="A87:G87"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A85:G85"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-16
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-15 10:01</t>
+          <t>Last updated: 2026-07-16 10:07</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1945,127 +1945,125 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 19:15_TAP_ret_TAP</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F44" s="6" t="n">
+      <c r="F45" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>247</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -2091,14 +2089,16 @@
       <c r="F49" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
@@ -2131,7 +2131,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -2164,7 +2164,7 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
@@ -2197,7 +2197,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -2230,7 +2230,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -2263,7 +2263,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -2452,16 +2452,16 @@
         </is>
       </c>
       <c r="F60" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G60" s="16" t="n">
-        <v>5</v>
+        <v>166</v>
+      </c>
+      <c r="G60" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="F61" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G61" s="15" t="n">
         <v>0</v>
@@ -2494,7 +2494,7 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -2520,14 +2520,14 @@
       <c r="F62" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
+      <c r="G62" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -2659,7 +2659,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2692,7 +2692,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -2782,16 +2782,16 @@
         </is>
       </c>
       <c r="F70" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G70" s="16" t="n">
-        <v>14</v>
+        <v>171</v>
+      </c>
+      <c r="G70" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="F71" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G71" s="15" t="n">
         <v>0</v>
@@ -2824,7 +2824,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -2850,14 +2850,14 @@
       <c r="F72" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G72" s="14" t="n">
-        <v>0</v>
+      <c r="G72" s="16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -2923,7 +2923,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -2956,7 +2956,7 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -2989,7 +2989,7 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -3022,7 +3022,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -3055,7 +3055,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -3088,7 +3088,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -3112,16 +3112,16 @@
         </is>
       </c>
       <c r="F80" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="G80" s="16" t="n">
-        <v>7</v>
+        <v>185</v>
+      </c>
+      <c r="G80" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="F81" s="6" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G81" s="15" t="n">
         <v>0</v>
@@ -3154,7 +3154,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -3180,56 +3180,113 @@
       <c r="F82" s="9" t="n">
         <v>192</v>
       </c>
-      <c r="G82" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
-        </is>
+      <c r="G82" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>192</v>
+      </c>
+      <c r="G83" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G84" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="F85" s="6" t="n">
-        <v>333</v>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
+        <v>192</v>
+      </c>
+      <c r="G85" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
@@ -3241,275 +3298,317 @@
       </c>
       <c r="B88" s="12" t="inlineStr">
         <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="n">
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G88" s="5" t="inlineStr">
+      <c r="G91" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="8" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B89" s="13" t="inlineStr">
+      <c r="B92" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
+      <c r="C92" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D89" s="8" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E89" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F89" s="9" t="n">
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G89" s="16" t="n">
+      <c r="G92" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="18" t="inlineStr">
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr">
+      <c r="E96" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F93" s="3" t="inlineStr">
+      <c r="F96" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G93" s="3" t="inlineStr">
+      <c r="G96" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E94" s="6" t="n">
+    <row r="97">
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="n">
         <v>167</v>
       </c>
-      <c r="F94" s="6" t="n">
+      <c r="F97" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G94" s="6" t="n">
-        <v>207.92</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="inlineStr">
+      <c r="G97" s="6" t="n">
+        <v>207.16</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B98" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr">
+      <c r="C98" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="D98" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E95" s="9" t="n">
+      <c r="E98" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="F95" s="9" t="n">
+      <c r="F98" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G95" s="9" t="n">
+      <c r="G98" s="9" t="n">
         <v>247</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="n">
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="F96" s="6" t="n">
+      <c r="F99" s="6" t="n">
         <v>192</v>
       </c>
-      <c r="G96" s="6" t="n">
-        <v>174.83</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="13" t="inlineStr">
+      <c r="G99" s="6" t="n">
+        <v>175.3</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B100" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr">
+      <c r="C100" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D97" s="8" t="inlineStr">
+      <c r="D100" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E97" s="9" t="n">
+      <c r="E100" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="F97" s="9" t="n">
+      <c r="F100" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="G97" s="9" t="n">
+      <c r="G100" s="9" t="n">
         <v>333</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="12" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B98" s="5" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
+      <c r="C101" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="n">
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="F98" s="6" t="n">
+      <c r="F101" s="6" t="n">
         <v>406</v>
       </c>
-      <c r="G98" s="6" t="n">
+      <c r="G101" s="6" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A87:G87"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A95:G95"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A90:G90"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3521,7 +3620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4748,1249 +4847,1247 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>246</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G48" s="16" t="n">
+      <c r="G49" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G55" s="15" t="n">
+      <c r="G56" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="G58" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G65" s="17" t="n">
+      <c r="G66" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="G68" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="G69" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="G70" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G70" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="G71" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="n">
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G71" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="G72" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G72" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+      <c r="G73" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="n">
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G73" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="G74" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="n">
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G74" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="G75" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F75" s="6" t="n">
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G75" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="G76" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B76" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F76" s="9" t="n">
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G76" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
+      <c r="G77" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="n">
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G77" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="G78" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G79" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B80" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F80" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G80" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F81" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G81" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
@@ -6014,16 +6111,18 @@
         </is>
       </c>
       <c r="F82" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G82" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
@@ -6047,189 +6146,288 @@
         </is>
       </c>
       <c r="F83" s="9" t="n">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>0</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G84" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="G85" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B84" s="12" t="inlineStr">
+      <c r="B86" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E84" s="5" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F84" s="6" t="n">
+      <c r="F86" s="6" t="n">
         <v>295</v>
       </c>
-      <c r="G84" s="17" t="n">
+      <c r="G86" s="17" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="18" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="n">
+        <v>269</v>
+      </c>
+      <c r="G87" s="14" t="n">
+        <v>-26</v>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr">
+      <c r="E91" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F88" s="3" t="inlineStr">
+      <c r="F91" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G88" s="3" t="inlineStr">
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E89" s="6" t="n">
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="F89" s="6" t="n">
+      <c r="F92" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G89" s="6" t="n">
-        <v>225.2</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D90" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E90" s="9" t="n">
+      <c r="G92" s="6" t="n">
+        <v>225.78</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="F90" s="9" t="n">
+      <c r="F93" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G90" s="9" t="n">
-        <v>215.2</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="12" t="inlineStr">
+      <c r="G93" s="9" t="n">
+        <v>215.53</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E91" s="6" t="n">
-        <v>280</v>
-      </c>
-      <c r="F91" s="6" t="n">
+      <c r="E94" s="6" t="n">
+        <v>269</v>
+      </c>
+      <c r="F94" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G91" s="6" t="n">
-        <v>298.4</v>
+      <c r="G94" s="6" t="n">
+        <v>293.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A81:G81"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A79:G79"/>
-    <mergeCell ref="A87:G87"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A90:G90"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-17
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-16 10:07</t>
+          <t>Last updated: 2026-07-17 09:55</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1978,160 +1978,158 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 19:15_TAP_ret_TAP</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F45" s="6" t="n">
+      <c r="F46" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F46" s="9" t="n">
+      <c r="F47" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>247</v>
+      </c>
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -2157,14 +2155,16 @@
       <c r="F51" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
@@ -2197,7 +2197,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -2230,7 +2230,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -2263,7 +2263,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -2296,7 +2296,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -2329,7 +2329,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -2494,7 +2494,7 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -2518,16 +2518,16 @@
         </is>
       </c>
       <c r="F62" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G62" s="16" t="n">
-        <v>5</v>
+        <v>166</v>
+      </c>
+      <c r="G62" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="F63" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G63" s="15" t="n">
         <v>0</v>
@@ -2560,7 +2560,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -2586,14 +2586,14 @@
       <c r="F64" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
+      <c r="G64" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -2659,7 +2659,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2692,7 +2692,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -2791,7 +2791,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2824,7 +2824,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -2848,16 +2848,16 @@
         </is>
       </c>
       <c r="F72" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G72" s="16" t="n">
-        <v>14</v>
+        <v>171</v>
+      </c>
+      <c r="G72" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="F73" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G73" s="15" t="n">
         <v>0</v>
@@ -2890,7 +2890,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -2916,14 +2916,14 @@
       <c r="F74" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G74" s="14" t="n">
-        <v>0</v>
+      <c r="G74" s="16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -2956,7 +2956,7 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -2989,7 +2989,7 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -3022,7 +3022,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -3055,7 +3055,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -3088,7 +3088,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -3121,7 +3121,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -3154,7 +3154,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -3178,16 +3178,16 @@
         </is>
       </c>
       <c r="F82" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="G82" s="16" t="n">
-        <v>7</v>
+        <v>185</v>
+      </c>
+      <c r="G82" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="F83" s="6" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G83" s="15" t="n">
         <v>0</v>
@@ -3220,7 +3220,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
@@ -3246,14 +3246,14 @@
       <c r="F84" s="9" t="n">
         <v>192</v>
       </c>
-      <c r="G84" s="14" t="n">
-        <v>0</v>
+      <c r="G84" s="16" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -3283,52 +3283,109 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
-        </is>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G86" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>192</v>
+      </c>
+      <c r="G87" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B88" s="12" t="inlineStr">
-        <is>
-          <t>21:55_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>21:55</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="n">
-        <v>333</v>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G88" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
@@ -3340,275 +3397,317 @@
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F91" s="6" t="n">
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G91" s="5" t="inlineStr">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="8" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B92" s="13" t="inlineStr">
+      <c r="B95" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C92" s="8" t="inlineStr">
+      <c r="C95" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D92" s="8" t="inlineStr">
+      <c r="D95" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E92" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F92" s="9" t="n">
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G92" s="16" t="n">
+      <c r="G95" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="18" t="inlineStr">
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr">
+      <c r="C99" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D96" s="3" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="E99" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F96" s="3" t="inlineStr">
+      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G96" s="3" t="inlineStr">
+      <c r="G99" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="n">
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="n">
         <v>167</v>
       </c>
-      <c r="F97" s="6" t="n">
+      <c r="F100" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G97" s="6" t="n">
-        <v>207.16</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="13" t="inlineStr">
+      <c r="G100" s="6" t="n">
+        <v>206.45</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
+      <c r="B101" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C98" s="8" t="inlineStr">
+      <c r="C101" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="D98" s="8" t="inlineStr">
+      <c r="D101" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E98" s="9" t="n">
+      <c r="E101" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="F98" s="9" t="n">
+      <c r="F101" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G98" s="9" t="n">
+      <c r="G101" s="9" t="n">
         <v>247</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="n">
+    <row r="102">
+      <c r="A102" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="F99" s="6" t="n">
+      <c r="F102" s="6" t="n">
         <v>192</v>
       </c>
-      <c r="G99" s="6" t="n">
-        <v>175.3</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="13" t="inlineStr">
+      <c r="G102" s="6" t="n">
+        <v>175.74</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="B103" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C100" s="8" t="inlineStr">
+      <c r="C103" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D100" s="8" t="inlineStr">
+      <c r="D103" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E100" s="9" t="n">
+      <c r="E103" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="F100" s="9" t="n">
+      <c r="F103" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="G100" s="9" t="n">
+      <c r="G103" s="9" t="n">
         <v>333</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="12" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B101" s="5" t="inlineStr">
+      <c r="B104" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E101" s="6" t="n">
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E104" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="F101" s="6" t="n">
+      <c r="F104" s="6" t="n">
         <v>406</v>
       </c>
-      <c r="G101" s="6" t="n">
+      <c r="G104" s="6" t="n">
         <v>385.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A93:G93"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A87:G87"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A95:G95"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A98:G98"/>
     <mergeCell ref="A90:G90"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A45:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3620,7 +3719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4880,1282 +4979,1280 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>255</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n">
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n">
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n">
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n">
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G49" s="16" t="n">
+      <c r="G50" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G51" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="n">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G52" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="G53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G53" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="G54" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="G55" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n">
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G55" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="n">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G56" s="15" t="n">
+      <c r="G57" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="n">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="G59" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="n">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="G61" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G61" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="n">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="G63" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G63" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="n">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G64" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="G65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G65" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G66" s="17" t="n">
+      <c r="G67" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="G69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="G70" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="n">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G70" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="G71" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G71" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
+      <c r="G72" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B72" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="n">
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G72" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="G73" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="n">
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G73" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+      <c r="G74" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B74" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F74" s="6" t="n">
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G74" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="G75" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="n">
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G75" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="5" t="inlineStr">
+      <c r="G76" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B76" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F76" s="6" t="n">
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G76" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="G77" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D77" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F77" s="9" t="n">
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G77" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
+      <c r="G78" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B78" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F78" s="6" t="n">
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G78" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="G79" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F79" s="9" t="n">
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G79" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="11" t="inlineStr">
+      <c r="G80" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="G81" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B82" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F82" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G82" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B83" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F83" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G83" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -6179,16 +6276,18 @@
         </is>
       </c>
       <c r="F84" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G84" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B85" s="13" t="inlineStr">
@@ -6212,16 +6311,16 @@
         </is>
       </c>
       <c r="F85" s="9" t="n">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>0</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -6245,189 +6344,255 @@
         </is>
       </c>
       <c r="F86" s="6" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G86" s="17" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="G87" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>295</v>
+      </c>
+      <c r="G88" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B87" s="13" t="inlineStr">
+      <c r="B89" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C87" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D87" s="8" t="inlineStr">
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E87" s="8" t="inlineStr">
+      <c r="E89" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F87" s="9" t="n">
+      <c r="F89" s="9" t="n">
         <v>269</v>
       </c>
-      <c r="G87" s="14" t="n">
+      <c r="G89" s="14" t="n">
         <v>-26</v>
       </c>
     </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="A90" s="18" t="inlineStr">
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B93" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C91" s="3" t="inlineStr">
+      <c r="C93" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D91" s="3" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr">
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F91" s="3" t="inlineStr">
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G91" s="3" t="inlineStr">
+      <c r="G93" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E92" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F92" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G92" s="6" t="n">
-        <v>225.78</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B93" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D93" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E93" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F93" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G93" s="9" t="n">
-        <v>215.53</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>255</v>
+      </c>
+      <c r="G94" s="6" t="n">
+        <v>226.57</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F95" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>215.84</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B94" s="5" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D94" s="5" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E94" s="6" t="n">
+      <c r="E96" s="6" t="n">
         <v>269</v>
       </c>
-      <c r="F94" s="6" t="n">
+      <c r="F96" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G94" s="6" t="n">
+      <c r="G96" s="6" t="n">
         <v>293.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A92:G92"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A90:G90"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily price update - 2026-07-18
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-17 09:55</t>
+          <t>Last updated: 2026-07-18 09:23</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2011,193 +2011,191 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 19:15_TAP_ret_TAP</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F46" s="6" t="n">
+      <c r="F47" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F47" s="9" t="n">
+      <c r="F48" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G47" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="F49" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G48" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>247</v>
+      </c>
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -2223,14 +2221,16 @@
       <c r="F53" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -2263,7 +2263,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -2296,7 +2296,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -2329,7 +2329,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -2494,7 +2494,7 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -2527,7 +2527,7 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -2584,16 +2584,16 @@
         </is>
       </c>
       <c r="F64" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G64" s="16" t="n">
-        <v>5</v>
+        <v>166</v>
+      </c>
+      <c r="G64" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="F65" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G65" s="15" t="n">
         <v>0</v>
@@ -2626,7 +2626,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -2652,14 +2652,14 @@
       <c r="F66" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
+      <c r="G66" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2692,7 +2692,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -2791,7 +2791,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2824,7 +2824,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -2857,7 +2857,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -2914,16 +2914,16 @@
         </is>
       </c>
       <c r="F74" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G74" s="16" t="n">
-        <v>14</v>
+        <v>171</v>
+      </c>
+      <c r="G74" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -2947,7 +2947,7 @@
         </is>
       </c>
       <c r="F75" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G75" s="15" t="n">
         <v>0</v>
@@ -2956,7 +2956,7 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -2982,14 +2982,14 @@
       <c r="F76" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G76" s="14" t="n">
-        <v>0</v>
+      <c r="G76" s="16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -3022,7 +3022,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -3055,7 +3055,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -3088,7 +3088,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -3121,7 +3121,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -3154,7 +3154,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -3187,7 +3187,7 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -3220,7 +3220,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
@@ -3244,16 +3244,16 @@
         </is>
       </c>
       <c r="F84" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="G84" s="16" t="n">
-        <v>7</v>
+        <v>185</v>
+      </c>
+      <c r="G84" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="F85" s="6" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G85" s="15" t="n">
         <v>0</v>
@@ -3286,7 +3286,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
@@ -3312,14 +3312,14 @@
       <c r="F86" s="9" t="n">
         <v>192</v>
       </c>
-      <c r="G86" s="14" t="n">
-        <v>0</v>
+      <c r="G86" s="16" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B87" s="12" t="inlineStr">
@@ -3352,7 +3352,7 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
@@ -3382,52 +3382,109 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
-        </is>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>192</v>
+      </c>
+      <c r="G89" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="G90" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t>21:55_BRI_ret_BRI</t>
+          <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>21:55</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="F91" s="6" t="n">
-        <v>333</v>
-      </c>
-      <c r="G91" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
+        <v>192</v>
+      </c>
+      <c r="G91" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_BRI</t>
         </is>
       </c>
     </row>
@@ -3439,262 +3496,304 @@
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
+          <t>21:55_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>21:55</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:55_BRI_ret_IBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D94" s="5" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F94" s="6" t="n">
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B95" s="13" t="inlineStr">
+      <c r="B98" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr">
+      <c r="C98" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="D98" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E95" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F95" s="9" t="n">
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="n">
         <v>406</v>
       </c>
-      <c r="G95" s="16" t="n">
+      <c r="G98" s="16" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="18" t="inlineStr">
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr">
+      <c r="C102" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D99" s="3" t="inlineStr">
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E99" s="3" t="inlineStr">
+      <c r="E102" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F99" s="3" t="inlineStr">
+      <c r="F102" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G99" s="3" t="inlineStr">
+      <c r="G102" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E100" s="6" t="n">
+    <row r="103">
+      <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="n">
         <v>167</v>
       </c>
-      <c r="F100" s="6" t="n">
+      <c r="F103" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="G100" s="6" t="n">
-        <v>206.45</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="13" t="inlineStr">
+      <c r="G103" s="6" t="n">
+        <v>205.77</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B104" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C101" s="8" t="inlineStr">
+      <c r="C104" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="D101" s="8" t="inlineStr">
+      <c r="D104" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E101" s="9" t="n">
+      <c r="E104" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="F101" s="9" t="n">
+      <c r="F104" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G101" s="9" t="n">
+      <c r="G104" s="9" t="n">
         <v>247</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E102" s="6" t="n">
+    <row r="105">
+      <c r="A105" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="F102" s="6" t="n">
+      <c r="F105" s="6" t="n">
         <v>192</v>
       </c>
-      <c r="G102" s="6" t="n">
-        <v>175.74</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="13" t="inlineStr">
+      <c r="G105" s="6" t="n">
+        <v>176.15</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="13" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B106" s="8" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C103" s="8" t="inlineStr">
+      <c r="C106" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D103" s="8" t="inlineStr">
+      <c r="D106" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E103" s="9" t="n">
+      <c r="E106" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="F103" s="9" t="n">
+      <c r="F106" s="9" t="n">
         <v>333</v>
       </c>
-      <c r="G103" s="9" t="n">
+      <c r="G106" s="9" t="n">
         <v>333</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="12" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="12" t="inlineStr">
         <is>
           <t>21:55_BRI_ret_IBE</t>
         </is>
       </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>21:55</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C107" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E104" s="6" t="n">
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="n">
         <v>365</v>
       </c>
-      <c r="F104" s="6" t="n">
+      <c r="F107" s="6" t="n">
         <v>406</v>
       </c>
-      <c r="G104" s="6" t="n">
+      <c r="G107" s="6" t="n">
         <v>385.5</v>
       </c>
     </row>
@@ -3702,12 +3801,12 @@
   <mergeCells count="8">
     <mergeCell ref="A93:G93"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A101:G101"/>
+    <mergeCell ref="A96:G96"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A52:G52"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A98:G98"/>
-    <mergeCell ref="A90:G90"/>
-    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3719,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5012,1315 +5111,1313 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>255</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G46" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G47" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G48" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="n">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G50" s="16" t="n">
+      <c r="G51" s="16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G52" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G53" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G53" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="G54" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G55" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="G56" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G56" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="n">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G57" s="15" t="n">
+      <c r="G58" s="15" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G58" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="n">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="G60" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G60" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="n">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="G62" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G62" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G63" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="G64" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G64" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="G66" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>206</v>
       </c>
-      <c r="G66" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="G67" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G67" s="17" t="n">
+      <c r="G68" s="17" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="G69" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="n">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="G70" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G70" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="G71" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="n">
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G71" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="G72" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G72" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+      <c r="G73" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="n">
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G73" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="G74" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="n">
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G74" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="G75" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F75" s="6" t="n">
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G75" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="G76" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B76" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F76" s="9" t="n">
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G76" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
+      <c r="G77" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="n">
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G77" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="G78" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="n">
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G78" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="inlineStr">
+      <c r="G79" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B79" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F79" s="6" t="n">
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G79" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="G80" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F80" s="9" t="n">
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="n">
         <v>227</v>
       </c>
-      <c r="G80" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
+      <c r="G81" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F81" s="6" t="n">
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G81" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="G82" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G83" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
         </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B84" s="12" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G84" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B85" s="13" t="inlineStr">
-        <is>
-          <t>21:35_BRI_ret_BRI</t>
-        </is>
-      </c>
-      <c r="C85" s="8" t="inlineStr">
-        <is>
-          <t>21:35</t>
-        </is>
-      </c>
-      <c r="D85" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>British Airways</t>
-        </is>
-      </c>
-      <c r="F85" s="9" t="n">
-        <v>280</v>
-      </c>
-      <c r="G85" s="14" t="n">
-        <v>-49</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -6344,16 +6441,18 @@
         </is>
       </c>
       <c r="F86" s="6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G86" s="17" t="n">
-        <v>14</v>
+        <v>329</v>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr">
@@ -6377,16 +6476,16 @@
         </is>
       </c>
       <c r="F87" s="9" t="n">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>0</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -6410,190 +6509,256 @@
         </is>
       </c>
       <c r="F88" s="6" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G88" s="17" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="G89" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="n">
+        <v>295</v>
+      </c>
+      <c r="G90" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B89" s="13" t="inlineStr">
+      <c r="B91" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
+      <c r="C91" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D89" s="8" t="inlineStr">
+      <c r="D91" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E89" s="8" t="inlineStr">
+      <c r="E91" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F89" s="9" t="n">
+      <c r="F91" s="9" t="n">
         <v>269</v>
       </c>
-      <c r="G89" s="14" t="n">
+      <c r="G91" s="14" t="n">
         <v>-26</v>
       </c>
     </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="18" t="inlineStr">
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B95" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr">
+      <c r="C95" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D95" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr">
+      <c r="E95" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F93" s="3" t="inlineStr">
+      <c r="F95" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G93" s="3" t="inlineStr">
+      <c r="G95" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E94" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="F94" s="6" t="n">
-        <v>255</v>
-      </c>
-      <c r="G94" s="6" t="n">
-        <v>226.57</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E95" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="F95" s="9" t="n">
-        <v>227</v>
-      </c>
-      <c r="G95" s="9" t="n">
-        <v>215.84</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
         <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="n">
+        <v>206</v>
+      </c>
+      <c r="F96" s="6" t="n">
+        <v>255</v>
+      </c>
+      <c r="G96" s="6" t="n">
+        <v>227.32</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="F97" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>216.13</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
+        <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B96" s="5" t="inlineStr">
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D96" s="5" t="inlineStr">
+      <c r="D98" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E96" s="6" t="n">
+      <c r="E98" s="6" t="n">
         <v>269</v>
       </c>
-      <c r="F96" s="6" t="n">
+      <c r="F98" s="6" t="n">
         <v>329</v>
       </c>
-      <c r="G96" s="6" t="n">
+      <c r="G98" s="6" t="n">
         <v>293.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A94:G94"/>
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A85:G85"/>
+    <mergeCell ref="A45:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update - 2026-07-19
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-18 09:23</t>
+          <t>Last updated: 2026-07-19 09:51</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2044,226 +2044,224 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 19:15_TAP_ret_TAP</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F47" s="6" t="n">
+      <c r="F48" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F48" s="9" t="n">
+      <c r="F49" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G48" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F49" s="6" t="n">
+      <c r="F50" s="6" t="n">
         <v>247</v>
       </c>
-      <c r="G49" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>19:15_TAP_ret_TAP</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="D50" s="8" t="inlineStr">
+      <c r="D51" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
         <is>
           <t>Tap Air Portugal</t>
         </is>
       </c>
-      <c r="F50" s="9" t="n">
+      <c r="F51" s="9" t="n">
         <v>247</v>
       </c>
-      <c r="G50" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>19:15_TAP_ret_TAP</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Tap Air Portugal</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>247</v>
+      </c>
+      <c r="G52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>166</v>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="G54" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -2289,14 +2287,16 @@
       <c r="F55" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -2329,7 +2329,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -2650,16 +2650,16 @@
         </is>
       </c>
       <c r="F66" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="G66" s="16" t="n">
-        <v>5</v>
+        <v>166</v>
+      </c>
+      <c r="G66" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2683,7 +2683,7 @@
         </is>
       </c>
       <c r="F67" s="6" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G67" s="15" t="n">
         <v>0</v>
@@ -2692,7 +2692,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -2718,14 +2718,14 @@
       <c r="F68" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="G68" s="14" t="n">
-        <v>0</v>
+      <c r="G68" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -2791,7 +2791,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2824,7 +2824,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -2857,7 +2857,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -2923,7 +2923,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -2956,7 +2956,7 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -2980,16 +2980,16 @@
         </is>
       </c>
       <c r="F76" s="9" t="n">
-        <v>185</v>
-      </c>
-      <c r="G76" s="16" t="n">
-        <v>14</v>
+        <v>171</v>
+      </c>
+      <c r="G76" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="F77" s="6" t="n">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="G77" s="15" t="n">
         <v>0</v>
@@ -3022,7 +3022,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -3048,14 +3048,14 @@
       <c r="F78" s="9" t="n">
         <v>185</v>
       </c>
-      <c r="G78" s="14" t="n">
-        <v>0</v>
+      <c r="G78" s="16" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -3088,7 +3088,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -3121,7 +3121,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -3154,7 +3154,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -3187,7 +3187,7 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -3220,7 +3220,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
@@ -3253,7 +3253,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -3286,7 +3286,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F86" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="G86" s="16" t="n">
-        <v>7</v>
+        <v>185</v>
+      </c>
+      <c r="G86" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>